<commit_message>
Revision: add OpenAlex, Crossref, update RWD, Scopus
</commit_message>
<xml_diff>
--- a/results/Table_1.xlsx
+++ b/results/Table_1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="95">
   <si>
     <t>Authors</t>
   </si>
@@ -85,6 +85,12 @@
     <t>Xiu et al.</t>
   </si>
   <si>
+    <t>Liu et al.</t>
+  </si>
+  <si>
+    <t>Li et al.</t>
+  </si>
+  <si>
     <t>2018 (2018)</t>
   </si>
   <si>
@@ -106,6 +112,12 @@
     <t>2023 (2023)</t>
   </si>
   <si>
+    <t>2024 (2024)</t>
+  </si>
+  <si>
+    <t>2025 (2025)</t>
+  </si>
+  <si>
     <t>Medical Physics</t>
   </si>
   <si>
@@ -148,6 +160,12 @@
     <t>Journal of Oncology</t>
   </si>
   <si>
+    <t>Neuroscience Informatics</t>
+  </si>
+  <si>
+    <t>Cancer Treatment and Research Communications</t>
+  </si>
+  <si>
     <t>WILEY</t>
   </si>
   <si>
@@ -157,6 +175,9 @@
     <t>Sage</t>
   </si>
   <si>
+    <t>Elsevier BV</t>
+  </si>
+  <si>
     <t>Iran</t>
   </si>
   <si>
@@ -272,6 +293,12 @@
   </si>
   <si>
     <t>10.1155/2023/8607062</t>
+  </si>
+  <si>
+    <t>10.1016/j.neuri.2024.100163</t>
+  </si>
+  <si>
+    <t>10.1016/j.ctarc.2025.100909</t>
   </si>
 </sst>
 </file>
@@ -629,7 +656,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -660,22 +687,22 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="F2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="G2" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -683,22 +710,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F3" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="G3" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -706,22 +733,22 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F4" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="G4" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -729,22 +756,22 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="F5" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="G5" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -752,22 +779,22 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="G6" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -775,22 +802,22 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F7" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="G7" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -798,22 +825,22 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="G8" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -821,22 +848,22 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="G9" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -844,22 +871,22 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="G10" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -867,22 +894,22 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="G11" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -890,22 +917,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="G12" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -913,22 +940,22 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E13" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F13" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="G13" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -936,22 +963,22 @@
         <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E14" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="G14" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -959,22 +986,22 @@
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E15" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F15" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="G15" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -982,22 +1009,22 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F16" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="G16" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1005,22 +1032,22 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E17" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F17" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="G17" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1028,22 +1055,22 @@
         <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D18" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="E18" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F18" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="G18" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1051,22 +1078,68 @@
         <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C19" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E19" t="s">
+        <v>55</v>
+      </c>
+      <c r="F19" t="s">
+        <v>74</v>
+      </c>
+      <c r="G19" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" t="s">
         <v>48</v>
       </c>
-      <c r="F19" t="s">
-        <v>67</v>
-      </c>
-      <c r="G19" t="s">
-        <v>85</v>
+      <c r="D20" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" t="s">
+        <v>74</v>
+      </c>
+      <c r="G20" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" t="s">
+        <v>58</v>
+      </c>
+      <c r="G21" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>